<commit_message>
Wire competitor density into volume engine + Excel
- keywordEngine: competition now = live competitor density per platform+keyword
  (from scrapes), driving Attack/Bid-up actions; threshold <12 = under-served
- Excel Rankings_Gaps: add competition band (Low/Med/High) + OPPORTUNITY flag
  (Low competition + you don't rank = easy win); 16 flagged

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qcomm-report.xlsx
+++ b/qcomm-report.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,24 +444,34 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>competition</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>competitors_seen</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>top_competitor</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>competitors_seen</t>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>OPPORTUNITY</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bagasse plates</t>
+          <t>banana leaf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -472,22 +482,30 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>fresho!</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>banana leaf</t>
+          <t>compostable containers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -498,22 +516,30 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>KCL Stainless</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Hazel</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>banana leaf plate</t>
+          <t>patravali</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -524,22 +550,30 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Banana Leaf</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>25</v>
+        <v>3</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bhandara plate</t>
+          <t>banana leaf plate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -550,22 +584,30 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sharda Metals</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Mad Over Print</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bhog plate</t>
+          <t>pattal</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -576,22 +618,30 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Shiv Shakti</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>biodegradable plates</t>
+          <t>sugarcane clamshell</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -602,50 +652,64 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Eco Aaroyaa</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TMI COLMAN</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>compostable containers</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>19</v>
-      </c>
+          <t>party plates</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>6</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>disposable banana leaf</t>
+          <t>snack plates</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -656,22 +720,30 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Natural Biodegradable</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>10</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Kitchen Essentials</t>
+        </is>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>disposable bowl</t>
+          <t>party tableware</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -682,22 +754,30 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Eco Disposable</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Eha Earth</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>disposable cup</t>
+          <t>sugarcane clamshell</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -708,22 +788,30 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Origami Disposable</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>25</v>
+        <v>2</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Forgreen Sugarcane</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>disposable plates</t>
+          <t>bhandara plate</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -734,22 +822,30 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>25</v>
+        <v>3</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Eha Earth</t>
+        </is>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>disposable plates for party</t>
+          <t>onam sadya plate</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -760,22 +856,30 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>25</v>
+        <v>3</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Eha Earth</t>
+        </is>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>disposable puja plate</t>
+          <t>biodegradable plates</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -786,22 +890,30 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Disposable Bagasse</t>
+        </is>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>disposable spoon</t>
+          <t>disposable banana leaf</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -812,50 +924,64 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Banana Stem</t>
+        </is>
+      </c>
+      <c r="H15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>disposable thali</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>22</v>
-      </c>
+          <t>disposable plates for party</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Eco Soul</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>24</v>
+        <v>9</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Disposable Bagasse</t>
+        </is>
+      </c>
+      <c r="H16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>amazon now</t>
+          <t>zepto</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>dona</t>
+          <t>sadhya leaf plate</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -866,11 +992,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>IAgriFarm 6</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>25</v>
+        <v>11</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Disposable Bagasse</t>
+        </is>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -881,7 +1015,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>eco friendly plates</t>
+          <t>patravali</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -892,11 +1026,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>25</v>
+        <v>19</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Silver Lord</t>
+        </is>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -907,22 +1049,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>katori</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>compostable containers</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>19</v>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CORELLE Herbs</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -933,22 +1085,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>modak plate</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>disposable thali</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>22</v>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aluminum Modak</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Eco Soul</t>
+        </is>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -959,7 +1121,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>onam sadya plate</t>
+          <t>bagasse plates</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -970,12 +1132,20 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Designer Brass</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>25</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -985,7 +1155,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>paper bowl</t>
+          <t>banana leaf</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -996,12 +1166,20 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Eco Aaroyaa</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>25</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>KCL Stainless</t>
+        </is>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1011,7 +1189,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>paper plate</t>
+          <t>banana leaf plate</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1022,12 +1200,20 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>25</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Banana Leaf</t>
+        </is>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1037,7 +1223,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>paper plates</t>
+          <t>bhandara plate</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1048,12 +1234,20 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>25</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Sharda Metals</t>
+        </is>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1063,7 +1257,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>party plates</t>
+          <t>bhog plate</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1074,12 +1268,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ECO SOUL</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>25</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Shiv Shakti</t>
+        </is>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1089,7 +1291,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>party tableware</t>
+          <t>biodegradable plates</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1100,12 +1302,20 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CELESTAIRE Premium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>25</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Eco Aaroyaa</t>
+        </is>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1115,7 +1325,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>patravali</t>
+          <t>disposable banana leaf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1126,11 +1336,19 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Silver Lord</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>19</v>
+        <v>25</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Natural Biodegradable</t>
+        </is>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1141,7 +1359,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>pattal</t>
+          <t>disposable bowl</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1152,12 +1370,20 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Brass Mart</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>25</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Eco Disposable</t>
+        </is>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1167,7 +1393,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>prasad bowl</t>
+          <t>disposable cup</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1178,12 +1404,20 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Auriant Brass</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>25</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Origami Disposable</t>
+        </is>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1193,7 +1427,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>prasad plate</t>
+          <t>disposable plates</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1204,12 +1438,20 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Shiv Shakti</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>25</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1219,7 +1461,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>puja thali</t>
+          <t>disposable plates for party</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1230,12 +1472,20 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BEHOMA Golden</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>25</v>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1245,7 +1495,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>sadhya leaf plate</t>
+          <t>disposable puja plate</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1256,12 +1506,20 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Palm Leaf</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>25</v>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1271,7 +1529,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>small bowl</t>
+          <t>disposable spoon</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1282,12 +1540,20 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>White Bone</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>25</v>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1297,7 +1563,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>snack plates</t>
+          <t>dona</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1308,12 +1574,20 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>miah decor</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F34" t="n">
         <v>25</v>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>IAgriFarm 6</t>
+        </is>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1323,7 +1597,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>sugarcane clamshell</t>
+          <t>eco friendly plates</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1334,12 +1608,20 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Disposable Bagasse</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>25</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1349,7 +1631,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>use and throw plate</t>
+          <t>katori</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1360,50 +1642,64 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Eco Soul</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>25</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>CORELLE Herbs</t>
+        </is>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>bagasse plates</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
-      </c>
+          <t>modak plate</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Classi Bio</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>15</v>
+        <v>25</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Aluminum Modak</t>
+        </is>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>banana leaf</t>
+          <t>onam sadya plate</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1414,22 +1710,30 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>fresho!</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5</v>
+        <v>25</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Designer Brass</t>
+        </is>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>biodegradable plates</t>
+          <t>paper bowl</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1440,22 +1744,30 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Origami</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Eco Aaroyaa</t>
+        </is>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>compostable containers</t>
+          <t>paper plate</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1466,50 +1778,64 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hazel</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>5</v>
+        <v>25</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H40" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>disposable bowl</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>6</v>
-      </c>
+          <t>paper plates</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Agrileaf</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>18</v>
+        <v>25</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H41" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>disposable cup</t>
+          <t>party plates</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1520,78 +1846,98 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>bb home</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>ECO SOUL</t>
+        </is>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>disposable plates</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>5</v>
-      </c>
+          <t>party tableware</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Agrileaf</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>14</v>
+        <v>25</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>CELESTAIRE Premium</t>
+        </is>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>disposable spoon</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>4</v>
-      </c>
+          <t>pattal</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Eco Soul</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>18</v>
+        <v>25</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Brass Mart</t>
+        </is>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>dona</t>
+          <t>prasad bowl</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1602,22 +1948,30 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>bb home</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Auriant Brass</t>
+        </is>
+      </c>
+      <c r="H45" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>eco friendly plates</t>
+          <t>prasad plate</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1628,22 +1982,30 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Agrileaf</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Shiv Shakti</t>
+        </is>
+      </c>
+      <c r="H46" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>katori</t>
+          <t>puja thali</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -1654,22 +2016,30 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Hazel</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>BEHOMA Golden</t>
+        </is>
+      </c>
+      <c r="H47" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>paper bowl</t>
+          <t>sadhya leaf plate</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -1680,22 +2050,30 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Nabhas</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Palm Leaf</t>
+        </is>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>paper plate</t>
+          <t>small bowl</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -1706,22 +2084,30 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Origami</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>White Bone</t>
+        </is>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>paper plates</t>
+          <t>snack plates</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -1732,50 +2118,64 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Origami</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>miah decor</t>
+        </is>
+      </c>
+      <c r="H50" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>party tableware</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>8</v>
-      </c>
+          <t>sugarcane clamshell</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Pasabahce</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>19</v>
+        <v>25</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Disposable Bagasse</t>
+        </is>
+      </c>
+      <c r="H51" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>bigbasket</t>
+          <t>amazon now</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>patravali</t>
+          <t>use and throw plate</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -1786,11 +2186,19 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>25</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
           <t>Eco Soul</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>20</v>
+      <c r="H52" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1801,22 +2209,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>pattal</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr"/>
+          <t>disposable plates</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>BB Royal Organic</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>20</v>
+        <v>14</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Agrileaf</t>
+        </is>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1827,22 +2245,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>small bowl</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
+          <t>bagasse plates</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Iveo</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Classi Bio</t>
+        </is>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1853,24 +2281,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>sugarcane clamshell</t>
+          <t>disposable bowl</t>
         </is>
       </c>
       <c r="C55" t="n">
+        <v>6</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ranked</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
         <v>18</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>ranked</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Nakoda</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
-        <v>19</v>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Agrileaf</t>
+        </is>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -1881,11 +2317,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>use and throw plate</t>
+          <t>disposable spoon</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1894,100 +2330,138 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Agrileaf</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Eco Soul</t>
+        </is>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>bagasse plates</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr"/>
+          <t>party tableware</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>8</v>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>14</v>
+        <v>19</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Pasabahce</t>
+        </is>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>banana leaf</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr"/>
+          <t>sugarcane clamshell</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>18</v>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Fruits and Vegetables</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>27</v>
+        <v>19</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Nakoda</t>
+        </is>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>banana leaf plate</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
+          <t>use and throw plate</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>6</v>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Mad Over Print</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>5</v>
+        <v>19</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Agrileaf</t>
+        </is>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>bhandara plate</t>
+          <t>biodegradable plates</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -1998,22 +2472,30 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Shri Samriddhi</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Origami</t>
+        </is>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>bhog plate</t>
+          <t>disposable cup</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -2024,50 +2506,64 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Sumeet</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>13</v>
+        <v>20</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>bb home</t>
+        </is>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>biodegradable plates</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>2</v>
-      </c>
+          <t>dona</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>13</v>
+        <v>20</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>bb home</t>
+        </is>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>compostable containers</t>
+          <t>eco friendly plates</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -2078,22 +2574,30 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Careswipe</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>12</v>
+        <v>20</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Agrileaf</t>
+        </is>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>disposable banana leaf</t>
+          <t>katori</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -2104,50 +2608,64 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>23</v>
+        <v>20</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Hazel</t>
+        </is>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>disposable bowl</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>1</v>
-      </c>
+          <t>paper bowl</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>16</v>
+        <v>20</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Nabhas</t>
+        </is>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>disposable cup</t>
+          <t>paper plate</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -2158,22 +2676,30 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Home Truths</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>16</v>
+        <v>20</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Origami</t>
+        </is>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>disposable plates</t>
+          <t>paper plates</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -2184,22 +2710,30 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Origami</t>
+        </is>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>disposable plates for party</t>
+          <t>patravali</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -2210,50 +2744,64 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Eco Soul</t>
+        </is>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>disposable puja plate</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>1</v>
-      </c>
+          <t>pattal</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Home Truths</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>31</v>
+        <v>20</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>BB Royal Organic</t>
+        </is>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>instamart</t>
+          <t>bigbasket</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>disposable spoon</t>
+          <t>small bowl</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -2264,11 +2812,19 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Home Truths</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>16</v>
+        <v>20</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Iveo</t>
+        </is>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2279,11 +2835,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>dona</t>
+          <t>party tableware</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2292,11 +2848,19 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Careswipe</t>
+        </is>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2307,7 +2871,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>eco friendly plates</t>
+          <t>dona</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -2320,11 +2884,19 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Origami</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -2335,7 +2907,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>katori</t>
+          <t>compostable containers</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -2346,11 +2918,19 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Haldiram's</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Careswipe</t>
+        </is>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2361,7 +2941,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>modak plate</t>
+          <t>bhog plate</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -2372,11 +2952,19 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Shri Samriddhi</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>20</v>
+        <v>13</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Sumeet</t>
+        </is>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2387,11 +2975,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>onam sadya plate</t>
+          <t>biodegradable plates</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -2400,11 +2988,19 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Shri Samriddhi</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>31</v>
+        <v>13</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -2415,24 +3011,30 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>paper bowl</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>1</v>
-      </c>
+          <t>bagasse plates</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>14</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
           <t>Ezee</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>16</v>
+      <c r="H76" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2443,7 +3045,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>paper plate</t>
+          <t>disposable plates</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -2454,12 +3056,20 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F77" t="n">
         <v>15</v>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2469,23 +3079,33 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>paper plates</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr"/>
+          <t>eco friendly plates</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F78" t="n">
         <v>15</v>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Origami</t>
+        </is>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2495,7 +3115,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>party plates</t>
+          <t>paper plate</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -2506,11 +3126,19 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>15</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
           <t>Ezee</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>6</v>
+      <c r="H79" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -2521,24 +3149,30 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>party tableware</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>2</v>
-      </c>
+          <t>paper plates</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ranked</t>
+          <t>GAP — not listed</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Careswipe</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>6</v>
+        <v>15</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2549,7 +3183,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>patravali</t>
+          <t>small bowl</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -2560,11 +3194,19 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Glass ideas</t>
+        </is>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -2575,7 +3217,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>pattal</t>
+          <t>use and throw plate</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -2586,11 +3228,19 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>15</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
           <t>Ezee</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>5</v>
+      <c r="H82" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -2601,22 +3251,32 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>puja thali</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr"/>
+          <t>disposable bowl</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Shri Samriddhi</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>33</v>
+        <v>16</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -2627,7 +3287,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>sadhya leaf plate</t>
+          <t>disposable cup</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -2638,11 +3298,19 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Ezee</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>20</v>
+        <v>16</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Home Truths</t>
+        </is>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -2653,7 +3321,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>small bowl</t>
+          <t>disposable spoon</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -2664,11 +3332,19 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Glass ideas</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Home Truths</t>
+        </is>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -2679,22 +3355,32 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>snack plates</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr"/>
+          <t>paper bowl</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1</v>
+      </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Kitchen Essentials</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -2705,7 +3391,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>sugarcane clamshell</t>
+          <t>bhandara plate</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -2716,11 +3402,19 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>TMI COLMAN</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>5</v>
+        <v>18</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Shri Samriddhi</t>
+        </is>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -2731,7 +3425,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>use and throw plate</t>
+          <t>disposable plates for party</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -2742,22 +3436,30 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>19</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
           <t>Ezee</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>15</v>
+      <c r="H88" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>bagasse plates</t>
+          <t>modak plate</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -2768,22 +3470,30 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Disposable Bagasse</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F89" t="n">
         <v>20</v>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Shri Samriddhi</t>
+        </is>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>banana leaf</t>
+          <t>sadhya leaf plate</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -2794,22 +3504,30 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Banana Leaves</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>banana leaf plate</t>
+          <t>katori</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -2820,22 +3538,30 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Disposable Bagasse</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Haldiram's</t>
+        </is>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>bhandara plate</t>
+          <t>disposable banana leaf</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -2846,22 +3572,30 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Eha Earth</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>3</v>
+        <v>23</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Ezee</t>
+        </is>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>biodegradable plates</t>
+          <t>banana leaf</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -2872,74 +3606,102 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Disposable Bagasse</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>5</v>
+        <v>27</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Fruits and Vegetables</t>
+        </is>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>disposable banana leaf</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr"/>
+          <t>disposable puja plate</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Banana Stem</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>6</v>
+        <v>31</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Home Truths</t>
+        </is>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>disposable bowl</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr"/>
+          <t>onam sadya plate</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>26</v>
+      </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>GAP — not listed</t>
+          <t>ranked</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Bagasse Bowl</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>21</v>
+        <v>31</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Shri Samriddhi</t>
+        </is>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>zepto</t>
+          <t>instamart</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>disposable cup</t>
+          <t>puja thali</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -2950,11 +3712,19 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Origami Disposable</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>16</v>
+        <v>33</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Shri Samriddhi</t>
+        </is>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -2965,7 +3735,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>disposable plates</t>
+          <t>dona</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -2976,11 +3746,19 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Disposable Paper</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>18</v>
+        <v>12</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Ezee Disposable</t>
+        </is>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -2991,7 +3769,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>disposable plates for party</t>
+          <t>disposable cup</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -3002,11 +3780,19 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Disposable Bagasse</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>9</v>
+        <v>16</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Origami Disposable</t>
+        </is>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -3017,7 +3803,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>disposable spoon</t>
+          <t>patravali</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -3028,11 +3814,19 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Tempware Wooden</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Marigold Yellow</t>
+        </is>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -3043,7 +3837,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>disposable thali</t>
+          <t>disposable plates</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -3054,11 +3848,19 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Round Disposable</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Disposable Paper</t>
+        </is>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -3069,7 +3871,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>dona</t>
+          <t>puja thali</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -3080,11 +3882,19 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Ezee Disposable</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>12</v>
+        <v>18</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Brass Pooja</t>
+        </is>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -3095,7 +3905,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>eco friendly plates</t>
+          <t>use and throw plate</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -3106,11 +3916,19 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Round Disposable</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F102" t="n">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Disposable Paper</t>
+        </is>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -3121,7 +3939,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>katori</t>
+          <t>bagasse plates</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
@@ -3132,11 +3950,19 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Bombay Kookware</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Disposable Bagasse</t>
+        </is>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -3147,7 +3973,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>onam sadya plate</t>
+          <t>disposable spoon</t>
         </is>
       </c>
       <c r="C104" t="inlineStr"/>
@@ -3158,11 +3984,19 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Eha Earth</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>3</v>
+        <v>20</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Tempware Wooden</t>
+        </is>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -3173,7 +4007,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>paper plate</t>
+          <t>disposable thali</t>
         </is>
       </c>
       <c r="C105" t="inlineStr"/>
@@ -3184,12 +4018,20 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Disposable Paper</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F105" t="n">
         <v>20</v>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Round Disposable</t>
+        </is>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3199,7 +4041,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>paper plates</t>
+          <t>paper plate</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -3210,12 +4052,20 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Disposable Paper</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F106" t="n">
         <v>20</v>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Disposable Paper</t>
+        </is>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3225,7 +4075,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>party plates</t>
+          <t>paper plates</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -3236,12 +4086,20 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Disposable Paper</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F107" t="n">
         <v>20</v>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Disposable Paper</t>
+        </is>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3251,7 +4109,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>party tableware</t>
+          <t>party plates</t>
         </is>
       </c>
       <c r="C108" t="inlineStr"/>
@@ -3262,11 +4120,19 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Eha Earth</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1</v>
+        <v>20</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Disposable Paper</t>
+        </is>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -3277,7 +4143,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>patravali</t>
+          <t>disposable bowl</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
@@ -3288,11 +4154,19 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Marigold Yellow</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F109" t="n">
-        <v>17</v>
+        <v>21</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Bagasse Bowl</t>
+        </is>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -3303,7 +4177,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>pattal</t>
+          <t>banana leaf plate</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -3314,11 +4188,19 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Bombay Kookware</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>25</v>
+        <v>22</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Disposable Bagasse</t>
+        </is>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -3329,7 +4211,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>prasad plate</t>
+          <t>eco friendly plates</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -3340,11 +4222,19 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Steelera Stainless</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>25</v>
+        <v>22</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Round Disposable</t>
+        </is>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -3355,7 +4245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>puja thali</t>
+          <t>banana leaf</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -3366,11 +4256,19 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Brass Pooja</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>18</v>
+        <v>25</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Banana Leaves</t>
+        </is>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -3381,7 +4279,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>sadhya leaf plate</t>
+          <t>katori</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
@@ -3392,11 +4290,19 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Disposable Bagasse</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>11</v>
+        <v>25</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Bombay Kookware</t>
+        </is>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -3407,7 +4313,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>snack plates</t>
+          <t>pattal</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -3418,12 +4324,20 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>The Earth</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F114" t="n">
         <v>25</v>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Bombay Kookware</t>
+        </is>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3433,7 +4347,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>sugarcane clamshell</t>
+          <t>prasad plate</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
@@ -3444,11 +4358,19 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Forgreen Sugarcane</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>2</v>
+        <v>25</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Steelera Stainless</t>
+        </is>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -3459,7 +4381,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>use and throw plate</t>
+          <t>snack plates</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -3470,11 +4392,19 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Disposable Paper</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>19</v>
+        <v>25</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>The Earth</t>
+        </is>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -76224,7 +77154,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>paper plate flowers</t>
+          <t>paper plates walmart</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -76240,7 +77170,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>paper plates walmart</t>
+          <t>paper plate awards</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -76256,7 +77186,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>paper plate animals</t>
+          <t>paper plates near me</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -76272,7 +77202,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>paper plates near me</t>
+          <t>paper plate dispenser</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -76288,7 +77218,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>paper plate dispenser</t>
+          <t>paper plate crafts</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -76304,7 +77234,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>paper plate crafts</t>
+          <t>paper plate flowers</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -76320,7 +77250,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>paper plate lion craft</t>
+          <t>paper plates bulk</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -76336,7 +77266,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>paper plates bulk</t>
+          <t>paper plates costco</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -76352,7 +77282,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>paper plates costco</t>
+          <t>paper plates in spanish</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -76400,7 +77330,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>paper plates in microwave</t>
+          <t>use and throw plates</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -76416,7 +77346,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>paper plates on sale</t>
+          <t>disposable cups with lids</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -76432,7 +77362,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>use and throw plates</t>
+          <t>disposable cup holders</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -76448,7 +77378,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>disposable cups with lids</t>
+          <t>disposable spoons</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -76464,7 +77394,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>disposable cup holder</t>
+          <t>disposable spoon rest</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -76480,7 +77410,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>disposable spoons</t>
+          <t>disposable spoon size</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -76496,7 +77426,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>disposable spoon rest</t>
+          <t>donald trump</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -76512,7 +77442,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>disposable spoon size</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -76528,7 +77458,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>donald trump</t>
+          <t>katori cutting board</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -76544,7 +77474,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>katori hall</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -76560,7 +77490,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>katori cutting board</t>
+          <t>katori bleach</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -76864,7 +77794,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>paper plate flowers</t>
+          <t>paper plates walmart</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -76880,7 +77810,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>paper plates walmart</t>
+          <t>paper plate awards</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -76896,7 +77826,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>paper plate animals</t>
+          <t>paper plates near me</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -76912,7 +77842,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>paper plates near me</t>
+          <t>paper plate dispenser</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -76928,7 +77858,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>paper plate dispenser</t>
+          <t>paper plate crafts</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -76944,7 +77874,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>paper plate crafts</t>
+          <t>paper plate flowers</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -76960,7 +77890,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>paper plate lion craft</t>
+          <t>paper plates bulk</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -76976,7 +77906,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>paper plates bulk</t>
+          <t>paper plates costco</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -76992,7 +77922,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>paper plates costco</t>
+          <t>paper plates in spanish</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -77040,7 +77970,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>paper plates in microwave</t>
+          <t>use and throw plates</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -77056,7 +77986,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>paper plates on sale</t>
+          <t>disposable cups with lids</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -77072,7 +78002,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>use and throw plates</t>
+          <t>disposable cup holders</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -77088,7 +78018,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>disposable cups with lids</t>
+          <t>disposable spoons</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -77104,7 +78034,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>disposable cup holder</t>
+          <t>disposable spoon rest</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -77120,7 +78050,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>disposable spoons</t>
+          <t>disposable spoon size</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -77136,7 +78066,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>disposable spoon rest</t>
+          <t>donald trump</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -77152,7 +78082,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>disposable spoon size</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -77168,7 +78098,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>donald trump</t>
+          <t>katori cutting board</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -77184,7 +78114,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>katori hall</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -77200,7 +78130,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>katori cutting board</t>
+          <t>katori bleach</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -78156,7 +79086,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>paper plate flowers</t>
+          <t>paper plates walmart</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
@@ -78172,7 +79102,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>paper plates walmart</t>
+          <t>paper plate awards</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -78188,7 +79118,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>paper plate animals</t>
+          <t>paper plates near me</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -78204,7 +79134,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>paper plates near me</t>
+          <t>paper plate dispenser</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
@@ -78220,7 +79150,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>paper plate dispenser</t>
+          <t>paper plate crafts</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -78236,7 +79166,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>paper plate crafts</t>
+          <t>paper plate flowers</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
@@ -78252,7 +79182,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>paper plate lion craft</t>
+          <t>paper plates bulk</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
@@ -78268,7 +79198,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>paper plates bulk</t>
+          <t>paper plates costco</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
@@ -78284,7 +79214,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>paper plates costco</t>
+          <t>paper plates in spanish</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
@@ -78332,7 +79262,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>paper plates in microwave</t>
+          <t>use and throw plates</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
@@ -78348,7 +79278,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>paper plates on sale</t>
+          <t>disposable cups with lids</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
@@ -78364,7 +79294,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>use and throw plates</t>
+          <t>disposable cup holders</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
@@ -78380,7 +79310,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>disposable cups with lids</t>
+          <t>disposable spoons</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
@@ -78396,7 +79326,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>disposable cup holder</t>
+          <t>disposable spoon rest</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
@@ -78412,7 +79342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>disposable spoons</t>
+          <t>disposable spoon size</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
@@ -78428,7 +79358,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>disposable spoon rest</t>
+          <t>donald trump</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
@@ -78444,7 +79374,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>disposable spoon size</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
@@ -78460,7 +79390,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>donald trump</t>
+          <t>katori cutting board</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -78476,7 +79406,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>katori hall</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -78492,7 +79422,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>katori cutting board</t>
+          <t>katori bleach</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -78796,7 +79726,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>paper plate flowers</t>
+          <t>paper plates walmart</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -78812,7 +79742,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>paper plates walmart</t>
+          <t>paper plate awards</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -78828,7 +79758,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>paper plate animals</t>
+          <t>paper plates near me</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
@@ -78844,7 +79774,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>paper plates near me</t>
+          <t>paper plate dispenser</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -78860,7 +79790,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>paper plate dispenser</t>
+          <t>paper plate crafts</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -78876,7 +79806,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>paper plate crafts</t>
+          <t>paper plate flowers</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -78892,7 +79822,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>paper plate lion craft</t>
+          <t>paper plates bulk</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -78908,7 +79838,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>paper plates bulk</t>
+          <t>paper plates costco</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
@@ -78924,7 +79854,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>paper plates costco</t>
+          <t>paper plates in spanish</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -78972,7 +79902,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>paper plates in microwave</t>
+          <t>use and throw plates</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -78988,7 +79918,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>paper plates on sale</t>
+          <t>disposable cups with lids</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
@@ -79004,7 +79934,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>use and throw plates</t>
+          <t>disposable cup holders</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
@@ -79020,7 +79950,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>disposable cups with lids</t>
+          <t>disposable spoons</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
@@ -79036,7 +79966,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>disposable cup holder</t>
+          <t>disposable spoon rest</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
@@ -79052,7 +79982,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>disposable spoons</t>
+          <t>disposable spoon size</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
@@ -79068,7 +79998,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>disposable spoon rest</t>
+          <t>donald trump</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
@@ -79084,7 +80014,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>disposable spoon size</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -79100,7 +80030,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>donald trump</t>
+          <t>katori cutting board</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -79116,7 +80046,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>katori hall</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -79132,7 +80062,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>katori cutting board</t>
+          <t>katori bleach</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
@@ -79436,7 +80366,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>paper plate flowers</t>
+          <t>paper plates walmart</t>
         </is>
       </c>
       <c r="C220" t="inlineStr"/>
@@ -79452,7 +80382,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>paper plates walmart</t>
+          <t>paper plate awards</t>
         </is>
       </c>
       <c r="C221" t="inlineStr"/>
@@ -79468,7 +80398,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>paper plate animals</t>
+          <t>paper plates near me</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
@@ -79484,7 +80414,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>paper plates near me</t>
+          <t>paper plate dispenser</t>
         </is>
       </c>
       <c r="C223" t="inlineStr"/>
@@ -79500,7 +80430,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>paper plate dispenser</t>
+          <t>paper plate crafts</t>
         </is>
       </c>
       <c r="C224" t="inlineStr"/>
@@ -79516,7 +80446,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>paper plate crafts</t>
+          <t>paper plate flowers</t>
         </is>
       </c>
       <c r="C225" t="inlineStr"/>
@@ -79532,7 +80462,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>paper plate lion craft</t>
+          <t>paper plates bulk</t>
         </is>
       </c>
       <c r="C226" t="inlineStr"/>
@@ -79548,7 +80478,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>paper plates bulk</t>
+          <t>paper plates costco</t>
         </is>
       </c>
       <c r="C227" t="inlineStr"/>
@@ -79564,7 +80494,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>paper plates costco</t>
+          <t>paper plates in spanish</t>
         </is>
       </c>
       <c r="C228" t="inlineStr"/>
@@ -79612,7 +80542,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>paper plates in microwave</t>
+          <t>use and throw plates</t>
         </is>
       </c>
       <c r="C231" t="inlineStr"/>
@@ -79628,7 +80558,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>paper plates on sale</t>
+          <t>disposable cups with lids</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
@@ -79644,7 +80574,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>use and throw plates</t>
+          <t>disposable cup holders</t>
         </is>
       </c>
       <c r="C233" t="inlineStr"/>
@@ -79660,7 +80590,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>disposable cups with lids</t>
+          <t>disposable spoons</t>
         </is>
       </c>
       <c r="C234" t="inlineStr"/>
@@ -79676,7 +80606,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>disposable cup holder</t>
+          <t>disposable spoon rest</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
@@ -79692,7 +80622,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>disposable spoons</t>
+          <t>disposable spoon size</t>
         </is>
       </c>
       <c r="C236" t="inlineStr"/>
@@ -79708,7 +80638,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>disposable spoon rest</t>
+          <t>donald trump</t>
         </is>
       </c>
       <c r="C237" t="inlineStr"/>
@@ -79724,7 +80654,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>disposable spoon size</t>
+          <t>katori titanium cutting board</t>
         </is>
       </c>
       <c r="C238" t="inlineStr"/>
@@ -79740,7 +80670,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>donald trump</t>
+          <t>katori cutting board</t>
         </is>
       </c>
       <c r="C239" t="inlineStr"/>
@@ -79756,7 +80686,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>katori titanium cutting board</t>
+          <t>katori hall</t>
         </is>
       </c>
       <c r="C240" t="inlineStr"/>
@@ -79772,7 +80702,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>katori cutting board</t>
+          <t>katori bleach</t>
         </is>
       </c>
       <c r="C241" t="inlineStr"/>

</xml_diff>